<commit_message>
GOTTA catch em all
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/demand_scenarios144.xlsx
+++ b/study_case_model/scenario_variables/demand_scenarios144.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>23906.58395364598</v>
+        <v>28725.35614758425</v>
       </c>
     </row>
     <row r="3">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2656.287105960664</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>9686.988486817821</v>
+        <v>23963.01774121611</v>
       </c>
     </row>
     <row r="6">
@@ -590,7 +590,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DORNUM</t>
+          <t>ST.FERGUS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>18516.93570487642</v>
+        <v>14928.8320178776</v>
       </c>
     </row>
     <row r="9">
@@ -611,7 +611,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DORNUM</t>
+          <t>ST.FERGUS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DORNUM</t>
+          <t>ST.FERGUS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>4629.233926219104</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -653,7 +653,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>39770.23628003302</v>
+        <v>29138.17913844815</v>
       </c>
     </row>
     <row r="12">
@@ -674,7 +674,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>7284.544784612039</v>
       </c>
     </row>
     <row r="14">
@@ -716,7 +716,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>8743.924962894067</v>
+        <v>46487.69937914996</v>
       </c>
     </row>
     <row r="15">
@@ -737,7 +737,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -775,11 +775,11 @@
         <v>2</v>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>20602.57302301981</v>
+        <v>11621.98641144057</v>
       </c>
     </row>
     <row r="18">
@@ -796,11 +796,11 @@
         <v>2</v>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2289.174780335534</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -817,11 +817,11 @@
         <v>2</v>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>38482.64895137142</v>
+        <v>36844.09611630544</v>
       </c>
     </row>
     <row r="21">
@@ -863,7 +863,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DORNUM</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>23845.05716760206</v>
+        <v>30755.76046864681</v>
       </c>
     </row>
     <row r="24">
@@ -926,7 +926,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DORNUM</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DORNUM</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -956,7 +956,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>5961.264291900515</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -968,7 +968,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>ST.FERGUS</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>41432.31515325805</v>
+        <v>10739.47105274393</v>
       </c>
     </row>
     <row r="27">
@@ -989,7 +989,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>ST.FERGUS</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>ST.FERGUS</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>14647.18543008559</v>
+        <v>23255.36026151579</v>
       </c>
     </row>
     <row r="30">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>5813.840065378947</v>
       </c>
     </row>
     <row r="32">
@@ -1090,11 +1090,11 @@
         <v>2</v>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>31945.64919695551</v>
+        <v>43048.73460781306</v>
       </c>
     </row>
     <row r="33">
@@ -1111,11 +1111,11 @@
         <v>2</v>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>3549.516577439501</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -1132,11 +1132,11 @@
         <v>2</v>
       </c>
       <c r="B34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1153,11 +1153,11 @@
         <v>2</v>
       </c>
       <c r="B35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>31934.75262184576</v>
+        <v>10753.51342411154</v>
       </c>
     </row>
     <row r="36">
@@ -1174,11 +1174,11 @@
         <v>2</v>
       </c>
       <c r="B36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1195,11 +1195,11 @@
         <v>2</v>
       </c>
       <c r="B37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>DORNUM</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>20357.78221952105</v>
+        <v>26814.71703674526</v>
       </c>
     </row>
     <row r="39">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>DORNUM</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>DORNUM</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1271,7 +1271,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>5089.445554880262</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>40295.94833441639</v>
+        <v>10650.39816506652</v>
       </c>
     </row>
     <row r="42">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>ST.FERGUS</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>15118.33742605096</v>
+        <v>6031.558128076127</v>
       </c>
     </row>
     <row r="45">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>ST.FERGUS</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>ST.FERGUS</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1405,11 +1405,11 @@
         <v>2</v>
       </c>
       <c r="B47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>25156.02635159681</v>
+        <v>16626.27482455417</v>
       </c>
     </row>
     <row r="48">
@@ -1426,11 +1426,11 @@
         <v>2</v>
       </c>
       <c r="B48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1439,7 +1439,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>2795.114039066312</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -1447,11 +1447,11 @@
         <v>2</v>
       </c>
       <c r="B49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ZEEBRUGGE</t>
+          <t>DORNUM</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0</v>
+        <v>4156.568706138542</v>
       </c>
     </row>
     <row r="50">
@@ -1468,11 +1468,11 @@
         <v>2</v>
       </c>
       <c r="B50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>31713.94915020799</v>
+        <v>34807.53319498364</v>
       </c>
     </row>
     <row r="51">
@@ -1489,11 +1489,11 @@
         <v>2</v>
       </c>
       <c r="B51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1510,11 +1510,11 @@
         <v>2</v>
       </c>
       <c r="B52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>EMDEN</t>
+          <t>DUNKERQUE</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1531,11 +1531,11 @@
         <v>2</v>
       </c>
       <c r="B53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>DORNUM</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>23811.03081009182</v>
+        <v>13678.42749723228</v>
       </c>
     </row>
     <row r="54">
@@ -1552,11 +1552,11 @@
         <v>2</v>
       </c>
       <c r="B54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>DORNUM</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1573,11 +1573,11 @@
         <v>2</v>
       </c>
       <c r="B55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>DORNUM</t>
+          <t>EASINGTON</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>5952.757702522955</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>65743.29072979002</v>
+        <v>18189.81943359092</v>
       </c>
     </row>
     <row r="57">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>DUNKERQUE</t>
+          <t>ZEEBRUGGE</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1670,7 +1670,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>10492.86795664787</v>
+        <v>14407.72223998532</v>
       </c>
     </row>
     <row r="60">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>EASINGTON</t>
+          <t>EMDEN</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1703,15 +1703,267 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
+          <t>EMDEN</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Vår Energi ASA</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B62" t="n">
+        <v>4</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ST.FERGUS</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Equinor Energy AS</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>17996.18288345583</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>2</v>
+      </c>
+      <c r="B63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>ST.FERGUS</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>SHELL</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>2</v>
+      </c>
+      <c r="B64" t="n">
+        <v>4</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>ST.FERGUS</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Vår Energi ASA</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>2</v>
+      </c>
+      <c r="B65" t="n">
+        <v>4</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>DORNUM</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Equinor Energy AS</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>18645.34219708079</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>2</v>
+      </c>
+      <c r="B66" t="n">
+        <v>4</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>DORNUM</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>SHELL</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>2</v>
+      </c>
+      <c r="B67" t="n">
+        <v>4</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>DORNUM</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Vår Energi ASA</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>4661.335549270197</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>2</v>
+      </c>
+      <c r="B68" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>DUNKERQUE</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Equinor Energy AS</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>51012.92307031886</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>2</v>
+      </c>
+      <c r="B69" t="n">
+        <v>4</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>DUNKERQUE</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>SHELL</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>2</v>
+      </c>
+      <c r="B70" t="n">
+        <v>4</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>DUNKERQUE</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Vår Energi ASA</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>2</v>
+      </c>
+      <c r="B71" t="n">
+        <v>4</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
           <t>EASINGTON</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Vår Energi ASA</t>
-        </is>
-      </c>
-      <c r="E61" t="n">
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Equinor Energy AS</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>7157.194301699537</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>2</v>
+      </c>
+      <c r="B72" t="n">
+        <v>4</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>EASINGTON</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>SHELL</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>2</v>
+      </c>
+      <c r="B73" t="n">
+        <v>4</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>EASINGTON</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Vår Energi ASA</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>